<commit_message>
added the unit of characterization column to the template to remind people what was chosen
</commit_message>
<xml_diff>
--- a/00_output/02_market_characterization.xlsx
+++ b/00_output/02_market_characterization.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,20 +513,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>characterization_unit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>single_family</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>multifamily</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>single_family_li</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>multifamily_li</t>
         </is>
@@ -543,6 +548,11 @@
           <t>oil_furnace</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>widget</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -555,6 +565,11 @@
           <t>gas_furnace</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>widget</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -565,6 +580,11 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>full_size</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>widget</t>
         </is>
       </c>
     </row>

</xml_diff>